<commit_message>
Added comments and added method to resolve path issue
</commit_message>
<xml_diff>
--- a/src/test/resources/testData/KODEXIQ_testData.xlsx
+++ b/src/test/resources/testData/KODEXIQ_testData.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Channambika\HSI_Training\KODEXIQ\KodexIQAutomation\KodexIQAutomationFrameworkDevelopment\src\test\resources\testData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7604E435-E69B-4B8A-A443-5F74D6152BC6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{131AD0C2-0109-4491-BEC4-78FBD7C22CC0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="36">
   <si>
     <t>username</t>
   </si>
@@ -105,13 +105,37 @@
   </si>
   <si>
     <t>Blank Password</t>
+  </si>
+  <si>
+    <t>PASS</t>
+  </si>
+  <si>
+    <t>2025-11-16 12:40:02</t>
+  </si>
+  <si>
+    <t>2025-11-16 12:40:13</t>
+  </si>
+  <si>
+    <t>2025-11-16 12:40:23</t>
+  </si>
+  <si>
+    <t>2025-11-16 12:40:34</t>
+  </si>
+  <si>
+    <t>2025-11-16 12:40:43</t>
+  </si>
+  <si>
+    <t>2025-11-16 12:40:54</t>
+  </si>
+  <si>
+    <t>2025-11-16 12:41:04</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -134,13 +158,53 @@
       <name val="Calibri"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color indexed="8"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color indexed="8"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color indexed="8"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color indexed="8"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color indexed="8"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color indexed="8"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color indexed="8"/>
+      <name val="Calibri"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor indexed="42"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="2">
@@ -171,7 +235,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -195,6 +259,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -508,7 +579,7 @@
     <col min="3" max="3" width="14.5546875" style="4" bestFit="1" customWidth="1" collapsed="1"/>
     <col min="4" max="4" width="33.109375" style="4" bestFit="1" customWidth="1" collapsed="1"/>
     <col min="5" max="5" width="8.88671875" style="4" collapsed="1"/>
-    <col min="6" max="6" width="11.109375" style="4" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="6" max="6" width="33.109375" style="4" bestFit="1" customWidth="1" collapsed="1"/>
     <col min="7" max="7" width="13.109375" style="4" bestFit="1" customWidth="1" collapsed="1"/>
     <col min="8" max="16384" width="8.88671875" style="4" collapsed="1"/>
   </cols>
@@ -549,9 +620,15 @@
       <c r="D2" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="E2" s="7"/>
-      <c r="F2" s="7"/>
-      <c r="G2" s="7"/>
+      <c r="E2" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="F2" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="G2" s="7" t="s">
+        <v>29</v>
+      </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" s="6" t="s">
@@ -562,9 +639,15 @@
       <c r="D3" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="E3" s="7"/>
-      <c r="F3" s="7"/>
-      <c r="G3" s="7"/>
+      <c r="E3" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="F3" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="G3" s="7" t="s">
+        <v>30</v>
+      </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" s="6" t="s">
@@ -577,9 +660,15 @@
       <c r="D4" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="E4" s="7"/>
-      <c r="F4" s="7"/>
-      <c r="G4" s="7"/>
+      <c r="E4" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="F4" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="G4" s="7" t="s">
+        <v>31</v>
+      </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" s="6" t="s">
@@ -592,9 +681,15 @@
       <c r="D5" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="E5" s="7"/>
-      <c r="F5" s="7"/>
-      <c r="G5" s="7"/>
+      <c r="E5" s="12" t="s">
+        <v>28</v>
+      </c>
+      <c r="F5" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="G5" s="7" t="s">
+        <v>32</v>
+      </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" s="6" t="s">
@@ -609,9 +704,15 @@
       <c r="D6" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="E6" s="7"/>
-      <c r="F6" s="7"/>
-      <c r="G6" s="7"/>
+      <c r="E6" s="13" t="s">
+        <v>28</v>
+      </c>
+      <c r="F6" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="G6" s="7" t="s">
+        <v>33</v>
+      </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" s="6" t="s">
@@ -626,9 +727,15 @@
       <c r="D7" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="E7" s="7"/>
-      <c r="F7" s="7"/>
-      <c r="G7" s="7"/>
+      <c r="E7" s="14" t="s">
+        <v>28</v>
+      </c>
+      <c r="F7" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="G7" s="7" t="s">
+        <v>34</v>
+      </c>
     </row>
     <row r="8" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A8" s="6" t="s">
@@ -643,9 +750,15 @@
       <c r="D8" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="E8" s="7"/>
-      <c r="F8" s="7"/>
-      <c r="G8" s="7"/>
+      <c r="E8" s="15" t="s">
+        <v>28</v>
+      </c>
+      <c r="F8" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="G8" s="7" t="s">
+        <v>35</v>
+      </c>
     </row>
   </sheetData>
   <hyperlinks>

</xml_diff>